<commit_message>
dados: incorpora conjuntos curados e sua classificacao
</commit_message>
<xml_diff>
--- a/nova_estetegia_levantamento/balanco_fase2_60_conjuntos.xlsx
+++ b/nova_estetegia_levantamento/balanco_fase2_60_conjuntos.xlsx
@@ -216,27 +216,27 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Nenhum concluído nesta etapa. D-001 foi preparado e aprovado na curadoria, mas aguarda check de instalação, integração e resposta dos autores. Não confundir aprovação de curadoria com permissão de redistribuição.</t>
+        <t>Nenhum concluído nesta etapa. D001 foi preparado e aprovado na curadoria, mas aguarda check de instalação, integração e resposta dos autores. Não confundir aprovação de curadoria com permissão de redistribuição.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D-001, D-002, ...; permanente após atribuição.</t>
+        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D001, D002, ...; permanente após atribuição.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D-001, D-002, ...; permanente após atribuição.</t>
+        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D001, D002, ...; permanente após atribuição.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D-001, D-002, ...; permanente após atribuição.</t>
+        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D001, D002, ...; permanente após atribuição.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D-001, D-002, ...; permanente após atribuição.</t>
+        <t>Apenas conjuntos com curadoria aprovada, documentação e validação concluídas. Cópias de treino e status antigos não significam incorporação concluída. Identificador no formato D001, D002, ...; permanente após atribuição.</t>
       </text>
     </comment>
   </commentList>
@@ -739,7 +739,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>D-001 bagre_racao_isoproteica: curadoria aprovada e integrado na main local da ClaRa em 11/10/2026. 200 testes passaram. Check de instalação e autorização dos autores pendentes; sem push. Dados prontos aguarda conclusão técnica formal.</t>
+          <t>D001 D001_bagre_racao_isoproteica: curadoria aprovada e integrado na main local da ClaRa em 11/10/2026. 200 testes passaram. Check de instalação e autorização dos autores pendentes; sem push. Dados prontos aguarda conclusão técnica formal.</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Ao concluir um conjunto, preencher de verde as células da linha correspondente em Núcleo 60 e Inventário e registrar conjunto, análises úteis, data e D-xxx em Dados prontos. Não alterar avaliações anteriores. D-xxx segue D-001, D-002, ...; códigos antigos L/E são preservados.</t>
+          <t>Ao concluir um conjunto, preencher de verde as células da linha correspondente em Núcleo 60 e Inventário e registrar conjunto, análises úteis, data e Dxxx em Dados prontos. Não alterar avaliações anteriores. Dxxx segue D001, D002, ...; códigos antigos L/E são preservados.</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Identificador ClaRa (D-xxx)</t>
+          <t>Identificador ClaRa (Dxx)</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -954,6 +954,16 @@
           <t>https://doi.org/10.17632/knsz9r4vby.5</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>D09</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="50.5" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -1022,6 +1032,16 @@
           <t>https://doi.org/10.5061/dryad.w3r2280ws</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="50.5" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1090,6 +1110,16 @@
           <t>https://stat.ethz.ch/R-manual/R-devel/library/datasets/html/Puromycin.html</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="50.5" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1162,6 +1192,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__bacteria.rda</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="50.5" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1230,6 +1270,16 @@
           <t>https://www.bco-dmo.org/dataset/724179/description</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="50.5" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1302,6 +1352,16 @@
           <t>R/data_abalone_adultos.R</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="50.5" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1374,6 +1434,16 @@
           <t>R/data_aquicultura_br.R</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="50.5" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1446,6 +1516,16 @@
           <t>R/data_bagley_lwr_central_america.R</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="50.5" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1518,6 +1598,16 @@
           <t>R/data_biometria_caranguejos.R</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="50.5" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1590,11 +1680,21 @@
           <t>R/data_brine_carbonatos.R</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="50.5" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>cabritos_fa_coltro</t>
+          <t xml:space="preserve">truta_acidos_graxos</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1604,17 +1704,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>PCA; HCA; comparação de dietas</t>
+          <t xml:space="preserve">PCA; HCA; exploração de dietas</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>precisa de ajuste</t>
+          <t xml:space="preserve">substituição aplicada</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Manter 32 animais e 10 colunas. n3/n6/sfa/mufa/pufa → omega_3_pct/omega_6_pct/saturados_pct/monoinsaturados_pct/poli_insaturados_pct; razões com prefixo razao_. T1…T4 → dieta_1…dieta_4, mantendo energia_mj_kg. Não inserir automaticamente razões junto com componentes na PCA.</t>
+          <t xml:space="preserve">Happel et al. (2021), Mendeley Data V2, CC BY 4.0. Semana 12: 60 peixes agregados em 21 aquários (UEs), três por dieta; 27 ácidos em porcentagem. Valor extremo mantido; sobrevivência baixa/desigual. Biplot aprovado como referência para reprodução futura em R.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1624,10 +1724,14 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
+          <t xml:space="preserve">Aprovar substituição</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Substituição dos cabritos por truta aprovada em 12/10/2026. Biplot aprovado pelo autor; reproduzir em R quando for feita a análise.</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Aprovar proposta</t>
@@ -1646,7 +1750,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>32 × 10</t>
+          <t xml:space="preserve">21 × 31</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1655,11 +1759,26 @@
         </is>
       </c>
       <c r="O12" s="2" t="n">
-        <v>2035</v>
+        <v>4728</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>R/data_cabritos_fa_coltro.R</t>
+          <t xml:space="preserve">R/data_truta_acidos_graxos.R</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D18: truta_acidos_graxos. Fonte original preservada, preparo R e médias conferidos. PCA: PC1 46,53%; PC2 21,74%.</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>D18</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12/10/2026</t>
         </is>
       </c>
     </row>
@@ -1734,6 +1853,16 @@
           <t>R/camarao_vannamei_biometria.R</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="50.5" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1806,6 +1935,16 @@
           <t>R/data_camaroes_sexo.R</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="50.5" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1878,6 +2017,16 @@
           <t>R/data_cangulo_crescimento.R</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="50.5" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1950,6 +2099,16 @@
           <t>R/data_captura_pescada_amarela.R; R/data_captura_pescada_amarela_bruta.R</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="50.5" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -2022,6 +2181,16 @@
           <t>R/data_captura_pescada_amarela_bruta.R</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="50.5" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -2094,6 +2263,16 @@
           <t>R/data_cpue_tubarao.R</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="50.5" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -2162,6 +2341,16 @@
         <v>1983</v>
       </c>
       <c r="P19" s="2" t="n"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="50.5" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2234,6 +2423,16 @@
           <t>R/data_darter_ontario.R</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="50.5" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -2306,6 +2505,16 @@
           <t>R/data_doubs_ambiente.R</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="50.5" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2378,6 +2587,16 @@
           <t>R/data_exportacao_pargo.R</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="50.5" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -2450,6 +2669,16 @@
           <t>R/data_gammarus_dieta_temperatura_resumo.R</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>D26</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="50.5" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -2522,6 +2751,16 @@
           <t>R/data_idades_savel_repetibilidade.R</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="50.5" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -2561,7 +2800,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>11/10/2026 — aprovado pelo autor no chat; solicitado preparo na ClaRa enquanto aguarda resposta dos autores. Objeto: bagre_racao_isoproteica; racao e peso_medio_final_g; 19 linhas preservadas. Autorização da fonte pendente. Check de instalação falhou também na ClaRa original; ainda não concluído.</t>
+          <t>11/10/2026 — aprovado pelo autor no chat; solicitado preparo na ClaRa enquanto aguarda resposta dos autores. Objeto: D001_bagre_racao_isoproteica; racao e peso_g; 19 linhas preservadas. Autorização da fonte pendente. Check de instalação falhou também na ClaRa original; ainda não concluído.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2600,12 +2839,12 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Integrado na main local; check e autorização da fonte pendentes</t>
+          <t>Integrado na main como D01; autorização da fonte pendente; check aprovado</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>D-001</t>
+          <t>D01</t>
         </is>
       </c>
     </row>
@@ -2680,6 +2919,16 @@
           <t>R/data_lagostas_kelp_sexo.R</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>D28</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="50.5" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -2752,6 +3001,16 @@
           <t>R/data_morfometria_barbo.R</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="50.5" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2824,6 +3083,16 @@
           <t>R/data_peixes_morfometria_multivariada.R</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>D29</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="50.5" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -2896,6 +3165,16 @@
           <t>R/data_peixes_nutricao_portugal.R</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>D30</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="50.5" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2968,6 +3247,16 @@
           <t>R/data_pinguins.R</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="50.5" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -3040,6 +3329,16 @@
           <t>R/qfasa_dados.R</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>D31</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="50.5" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -3112,6 +3411,16 @@
           <t>R/qfasa_dados.R</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>D32</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="50.5" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
@@ -3184,6 +3493,16 @@
           <t>R/data_recifes_ostras_heatmap.R</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>D33</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="50.5" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -3256,6 +3575,16 @@
           <t>R/data_salvelino_formalina_remocao.R</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="50.5" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -3324,6 +3653,16 @@
         <v>2448</v>
       </c>
       <c r="P35" s="2" t="n"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="50.5" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -3396,6 +3735,16 @@
           <t>R/data_tilapia_microalgas.R</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>D35</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="50.5" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
@@ -3468,6 +3817,16 @@
           <t>R/data_treino_coletas.R</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>D36</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="50.5" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -3540,6 +3899,16 @@
           <t>R/data_treino_desembarque.R</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>D37</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="50.5" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -3612,6 +3981,16 @@
           <t>R/data_truta_riacho_crescimento.R</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>D38</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="50.5" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -3680,6 +4059,16 @@
         <v>123634</v>
       </c>
       <c r="P40" s="2" t="n"/>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Revisado; colunas e categorias aprovadas; integrado na main; check aprovado; colunas e categorias aprovadas; comprimento do registro 234 a conferir; usar massa inicialmente; substituído por cowichan_amostragem</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>D39</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="50.5" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -3752,6 +4141,16 @@
           <t>https://doi.org/10.5061/dryad.bg79cnpph</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>D40</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="50.5" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -3824,6 +4223,16 @@
           <t>https://doi.org/10.5061/dryad.hx3ffbgkn</t>
         </is>
       </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="50.5" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -3892,6 +4301,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__PlantGrowth.rda</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>D42</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="50.5" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -3960,6 +4379,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__npk.rda</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>D43</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="50.5" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
@@ -4028,6 +4457,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__CO2.rda</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>D44</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="50.5" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -4100,6 +4539,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__InsectSprays.rda</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>D45</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="50.5" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -4168,6 +4617,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__cars.rda</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>D46</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="50.5" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -4240,6 +4699,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__quakes.rda</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="50.5" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -4312,6 +4781,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__Orange.rda</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>D48</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="50.5" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -4380,6 +4859,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__oats.rda</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="50.5" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -4448,6 +4937,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__quine.rda</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>D50 substituído por molinesias_parasitos (Dryad CC0), autorizado em 11/10/2026; 128 peixes, 8 colunas; check aprovado; curadoria fina provisória; fonte quine preservada no histórico</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>D50</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="50.5" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -4516,6 +5015,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__Insurance.rda</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>D51</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="50.5" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
@@ -4584,6 +5093,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__wtloss.rda</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="50.5" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -4656,6 +5175,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__ships.rda</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>D53</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="50.5" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
@@ -4724,6 +5253,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__WhiteGrunt2.rda</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>D54</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="50.5" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -4792,6 +5331,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__Cabezon.rda</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>D55</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="50.5" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -4860,6 +5409,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__RuffeSLRH92.rda</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>D56</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="50.5" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -4928,6 +5487,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__BGHRsample.rda</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="50.5" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -4996,6 +5565,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__BGHRfish.rda</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>D58</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="50.5" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -5064,6 +5643,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/astsa__rec.rda</t>
         </is>
       </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>D59</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="50.5" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -5130,6 +5719,16 @@
       <c r="P61" s="2" t="inlineStr">
         <is>
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/agridat__cochran.latin.rda</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>D60</t>
         </is>
       </c>
     </row>
@@ -5258,7 +5857,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Identificador ClaRa (D-xxx)</t>
+          <t>Identificador ClaRa (Dxx)</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -5334,6 +5933,16 @@
           <t>https://doi.org/10.17632/knsz9r4vby.5</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>D09</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="95" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -5402,6 +6011,16 @@
           <t>https://doi.org/10.5061/dryad.w3r2280ws</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="95" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -5470,6 +6089,16 @@
           <t>https://stat.ethz.ch/R-manual/R-devel/library/datasets/html/Puromycin.html</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="95" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -5542,6 +6171,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__bacteria.rda</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="95" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -5610,6 +6249,16 @@
           <t>https://www.bco-dmo.org/dataset/724179/description</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="95" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -5682,6 +6331,16 @@
           <t>R/data_abalone_adultos.R</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="95" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -5754,6 +6413,16 @@
           <t>R/data_aquicultura_br.R</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="95" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -5902,6 +6571,16 @@
           <t>R/data_bagley_lwr_central_america.R</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="95" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -5974,6 +6653,16 @@
           <t>R/data_biometria_caranguejos.R</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="95" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -6046,11 +6735,21 @@
           <t>R/data_brine_carbonatos.R</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>cabritos_fa_coltro</t>
+          <t xml:space="preserve">truta_acidos_graxos</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -6060,17 +6759,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>PCA; HCA; comparação de dietas</t>
+          <t xml:space="preserve">PCA; HCA; exploração de dietas</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>precisa de ajuste</t>
+          <t xml:space="preserve">substituição aplicada</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Manter 32 animais e 10 colunas. n3/n6/sfa/mufa/pufa → omega_3_pct/omega_6_pct/saturados_pct/monoinsaturados_pct/poli_insaturados_pct; razões com prefixo razao_. T1…T4 → dieta_1…dieta_4, mantendo energia_mj_kg. Não inserir automaticamente razões junto com componentes na PCA.</t>
+          <t xml:space="preserve">Happel et al. (2021), Mendeley Data V2, CC BY 4.0. Semana 12: 60 peixes agregados em 21 aquários (UEs), três por dieta; 27 ácidos em porcentagem. Valor extremo mantido; sobrevivência baixa/desigual. Biplot aprovado como referência para reprodução futura em R.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -6080,10 +6779,14 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="n"/>
+          <t xml:space="preserve">Aprovar substituição</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Substituição dos cabritos por truta aprovada em 12/10/2026. Biplot aprovado pelo autor; reproduzir em R quando for feita a análise.</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Aprovar proposta</t>
@@ -6102,7 +6805,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>32 × 10</t>
+          <t xml:space="preserve">21 × 31</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -6111,11 +6814,26 @@
         </is>
       </c>
       <c r="O13" s="2" t="n">
-        <v>2035</v>
+        <v>4728</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>R/data_cabritos_fa_coltro.R</t>
+          <t xml:space="preserve">R/data_truta_acidos_graxos.R</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D18: truta_acidos_graxos. Fonte original preservada, preparo R e médias conferidos. PCA: PC1 46,53%; PC2 21,74%.</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>D18</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12/10/2026</t>
         </is>
       </c>
     </row>
@@ -6190,6 +6908,16 @@
           <t>R/camarao_vannamei_biometria.R</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="95" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -6262,6 +6990,16 @@
           <t>R/data_camaroes_sexo.R</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="95" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -6334,6 +7072,16 @@
           <t>R/data_cangulo_crescimento.R</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="95" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -6406,6 +7154,16 @@
           <t>R/data_captura_pescada_amarela.R; R/data_captura_pescada_amarela_bruta.R</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="95" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -6478,6 +7236,16 @@
           <t>R/data_captura_pescada_amarela_bruta.R</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="95" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -6622,6 +7390,16 @@
           <t>R/data_cpue_tubarao.R</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="95" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -6690,6 +7468,16 @@
         <v>1983</v>
       </c>
       <c r="P21" s="2" t="n"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="95" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -6762,6 +7550,16 @@
           <t>R/data_darter_ontario.R</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="95" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -6902,6 +7700,16 @@
           <t>R/data_doubs_ambiente.R</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="95" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -7046,6 +7854,16 @@
           <t>R/data_exportacao_pargo.R</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="95" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -7118,6 +7936,16 @@
           <t>R/data_gammarus_dieta_temperatura_resumo.R</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>D26</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="95" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -7190,6 +8018,16 @@
           <t>R/data_idades_savel_repetibilidade.R</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="95" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -7229,7 +8067,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>11/10/2026 — aprovado pelo autor no chat; solicitado preparo na ClaRa enquanto aguarda resposta dos autores. Objeto: bagre_racao_isoproteica; racao e peso_medio_final_g; 19 linhas preservadas. Autorização da fonte pendente. Check de instalação falhou também na ClaRa original; ainda não concluído.</t>
+          <t>11/10/2026 — aprovado pelo autor no chat; solicitado preparo na ClaRa enquanto aguarda resposta dos autores. Objeto: D001_bagre_racao_isoproteica; racao e peso_g; 19 linhas preservadas. Autorização da fonte pendente. Check de instalação falhou também na ClaRa original; ainda não concluído.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -7268,12 +8106,12 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Integrado na main local; check e autorização da fonte pendentes</t>
+          <t>Integrado na main como D01; autorização da fonte pendente; check aprovado</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>D-001</t>
+          <t>D01</t>
         </is>
       </c>
     </row>
@@ -7348,6 +8186,16 @@
           <t>R/data_lagostas_kelp_sexo.R</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>D28</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="95" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -7420,6 +8268,16 @@
           <t>R/data_morfometria_barbo.R</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="95" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -7564,6 +8422,16 @@
           <t>R/data_peixes_morfometria_multivariada.R</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>D29</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="95" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -7636,6 +8504,16 @@
           <t>R/data_peixes_nutricao_portugal.R</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>D30</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="95" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -7708,6 +8586,16 @@
           <t>R/data_pinguins.R</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="95" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -7852,6 +8740,16 @@
           <t>R/qfasa_dados.R</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>D31</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="95" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -7924,6 +8822,16 @@
           <t>R/qfasa_dados.R</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>D32</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="95" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -7996,6 +8904,16 @@
           <t>R/data_recifes_ostras_heatmap.R</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>D33</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="95" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -8136,6 +9054,16 @@
           <t>R/data_salvelino_formalina_remocao.R</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="95" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -8204,6 +9132,16 @@
         <v>2448</v>
       </c>
       <c r="P42" s="2" t="n"/>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="95" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -8420,6 +9358,16 @@
           <t>R/data_tilapia_microalgas.R</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>D35</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="95" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -8492,6 +9440,16 @@
           <t>R/data_treino_coletas.R</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>D36</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="95" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -8564,6 +9522,16 @@
           <t>R/data_treino_desembarque.R</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>D37</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="95" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -8636,6 +9604,16 @@
           <t>R/data_truta_riacho_crescimento.R</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>D38</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="95" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -8704,6 +9682,16 @@
         <v>123634</v>
       </c>
       <c r="P49" s="2" t="n"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Revisado; colunas e categorias aprovadas; integrado na main; check aprovado; colunas e categorias aprovadas; comprimento do registro 234 a conferir; usar massa inicialmente; substituído por cowichan_amostragem</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>D39</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="95" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -8776,6 +9764,16 @@
           <t>https://doi.org/10.5061/dryad.bg79cnpph</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>D40</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="95" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -8848,6 +9846,16 @@
           <t>https://doi.org/10.5061/dryad.hx3ffbgkn</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="95" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -8916,6 +9924,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__PlantGrowth.rda</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>D42</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="95" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
@@ -8984,6 +10002,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__npk.rda</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>D43</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="95" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -9468,6 +10496,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__CO2.rda</t>
         </is>
       </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>D44</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="95" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -9540,6 +10578,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__InsectSprays.rda</t>
         </is>
       </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>D45</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="95" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -9676,6 +10724,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__cars.rda</t>
         </is>
       </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>D46</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="95" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -9884,6 +10942,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__quakes.rda</t>
         </is>
       </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="95" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
@@ -9956,6 +11024,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/datasets__Orange.rda</t>
         </is>
       </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>D48</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="95" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -10168,6 +11246,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__oats.rda</t>
         </is>
       </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="95" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
@@ -10304,6 +11392,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__quine.rda</t>
         </is>
       </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>D50 substituído por molinesias_parasitos (Dryad CC0), autorizado em 11/10/2026; 128 peixes, 8 colunas; check aprovado; curadoria fina provisória; fonte quine preservada no histórico</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>D50</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="95" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
@@ -10372,6 +11470,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__Insurance.rda</t>
         </is>
       </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>D51</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="95" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
@@ -10440,6 +11548,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__wtloss.rda</t>
         </is>
       </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="95" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
@@ -10512,6 +11630,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/MASS__ships.rda</t>
         </is>
       </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>D53</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="95" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
@@ -10784,6 +11912,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__WhiteGrunt2.rda</t>
         </is>
       </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>D54</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="95" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
@@ -10852,6 +11990,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__Cabezon.rda</t>
         </is>
       </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>D55</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="95" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
@@ -10920,6 +12068,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__RuffeSLRH92.rda</t>
         </is>
       </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>D56</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="95" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
@@ -10988,6 +12146,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__BGHRsample.rda</t>
         </is>
       </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="95" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
@@ -11056,6 +12224,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/FSAdata__BGHRfish.rda</t>
         </is>
       </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>D58</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="95" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
@@ -11668,6 +12846,16 @@
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/astsa__rec.rda</t>
         </is>
       </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>D59</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="95" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
@@ -11802,6 +12990,16 @@
       <c r="P94" s="2" t="inlineStr">
         <is>
           <t>D:/Claude/EAPA-Ecossistema/EAPADados/nova_estetegia_levantamento/levantamento_tecnico/objetos_originais/agridat__cochran.latin.rda</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Passada 1 provisória integrada na main; check aprovado; curadoria pendente</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>D60</t>
         </is>
       </c>
     </row>
@@ -13317,7 +14515,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Identificador (D-xxx)</t>
+          <t>Identificador (Dxxx)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">

</xml_diff>